<commit_message>
adds large nuclear tyche style data
</commit_message>
<xml_diff>
--- a/src/technology/small-modular-reactor/small-modular-reactor-fixed.xlsx
+++ b/src/technology/small-modular-reactor/small-modular-reactor-fixed.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhanes\GitHub\tyche\src\technology\small-modular-reactor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777E9D14-4757-4AC6-8FF8-270A8D9054E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B066BC-FD87-49E4-9C73-C2F411D9603B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17070" yWindow="2415" windowWidth="27015" windowHeight="16755" tabRatio="778" activeTab="8" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
+    <workbookView xWindow="6420" yWindow="90" windowWidth="19425" windowHeight="20805" tabRatio="778" activeTab="4" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
   </bookViews>
   <sheets>
     <sheet name="indices" sheetId="1" r:id="rId1"/>
@@ -24,9 +24,10 @@
     <sheet name="investments" sheetId="7" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">designs!$A$1:$G$890</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indices!$A$1:$F$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">parameters!$A$1:$G$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">designs!$A$1:$G$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indices!$A$1:$F$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">parameters!$A$1:$G$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">results!$A$1:$E$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2167" uniqueCount="141">
   <si>
     <t>Category</t>
   </si>
@@ -457,16 +458,37 @@
   </si>
   <si>
     <t>Total OCC</t>
+  </si>
+  <si>
+    <t>Large Nuclear</t>
+  </si>
+  <si>
+    <t>reactor_type</t>
+  </si>
+  <si>
+    <t>1 = Concept A, Large Nuclear; 0 = Concept B, Small Modular Reactor</t>
+  </si>
+  <si>
+    <t>Variable Op and Maint</t>
+  </si>
+  <si>
+    <t>Fixed Op and Maint</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -808,7 +830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF3D170-DEC1-4938-B961-67DBF048922E}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -928,20 +950,174 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C10" t="s">
         <v>100</v>
       </c>
-      <c r="D8">
+      <c r="D10">
         <v>0</v>
       </c>
     </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>102</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>136</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>135</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>139</v>
+      </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>140</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F25">
-    <sortCondition ref="A3:A25"/>
-    <sortCondition ref="B3:B25"/>
-    <sortCondition ref="D3:D25"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F29">
+    <sortCondition ref="A3:A29"/>
+    <sortCondition ref="B3:B29"/>
+    <sortCondition ref="D3:D29"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1018,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A97C873A-D063-4744-8651-CEF648C63973}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -1083,6 +1259,32 @@
         <v>36</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1090,7 +1292,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FB20890-62B7-47AF-BA68-650F053D99C5}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -1965,7 +2167,848 @@
         <v>104</v>
       </c>
     </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>136</v>
+      </c>
+      <c r="B44" t="s">
+        <v>71</v>
+      </c>
+      <c r="C44" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" t="s">
+        <v>99</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="F44" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>136</v>
+      </c>
+      <c r="B45" t="s">
+        <v>71</v>
+      </c>
+      <c r="C45" t="s">
+        <v>29</v>
+      </c>
+      <c r="D45" t="s">
+        <v>99</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="F45" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>136</v>
+      </c>
+      <c r="B46" t="s">
+        <v>71</v>
+      </c>
+      <c r="C46" t="s">
+        <v>32</v>
+      </c>
+      <c r="D46" t="s">
+        <v>99</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>136</v>
+      </c>
+      <c r="B47" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" t="s">
+        <v>34</v>
+      </c>
+      <c r="D47" t="s">
+        <v>98</v>
+      </c>
+      <c r="E47">
+        <v>50</v>
+      </c>
+      <c r="F47" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>136</v>
+      </c>
+      <c r="B48" t="s">
+        <v>71</v>
+      </c>
+      <c r="C48" t="s">
+        <v>30</v>
+      </c>
+      <c r="D48" t="s">
+        <v>100</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>136</v>
+      </c>
+      <c r="B49" t="s">
+        <v>71</v>
+      </c>
+      <c r="C49" t="s">
+        <v>33</v>
+      </c>
+      <c r="D49" t="s">
+        <v>100</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>136</v>
+      </c>
+      <c r="B50" t="s">
+        <v>71</v>
+      </c>
+      <c r="C50" t="s">
+        <v>31</v>
+      </c>
+      <c r="D50" t="s">
+        <v>98</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+      <c r="F50" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>136</v>
+      </c>
+      <c r="B51" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" t="s">
+        <v>99</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>136</v>
+      </c>
+      <c r="B52" t="s">
+        <v>88</v>
+      </c>
+      <c r="C52" t="s">
+        <v>29</v>
+      </c>
+      <c r="D52" t="s">
+        <v>99</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>136</v>
+      </c>
+      <c r="B53" t="s">
+        <v>88</v>
+      </c>
+      <c r="C53" t="s">
+        <v>32</v>
+      </c>
+      <c r="D53" t="s">
+        <v>99</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>136</v>
+      </c>
+      <c r="B54" t="s">
+        <v>88</v>
+      </c>
+      <c r="C54" t="s">
+        <v>34</v>
+      </c>
+      <c r="D54" t="s">
+        <v>98</v>
+      </c>
+      <c r="E54">
+        <v>50</v>
+      </c>
+      <c r="F54" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>136</v>
+      </c>
+      <c r="B55" t="s">
+        <v>88</v>
+      </c>
+      <c r="C55" t="s">
+        <v>30</v>
+      </c>
+      <c r="D55" t="s">
+        <v>100</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>136</v>
+      </c>
+      <c r="B56" t="s">
+        <v>88</v>
+      </c>
+      <c r="C56" t="s">
+        <v>33</v>
+      </c>
+      <c r="D56" t="s">
+        <v>100</v>
+      </c>
+      <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="F56" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>136</v>
+      </c>
+      <c r="B57" t="s">
+        <v>88</v>
+      </c>
+      <c r="C57" t="s">
+        <v>31</v>
+      </c>
+      <c r="D57" t="s">
+        <v>98</v>
+      </c>
+      <c r="E57">
+        <v>1</v>
+      </c>
+      <c r="F57" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>136</v>
+      </c>
+      <c r="B58" t="s">
+        <v>87</v>
+      </c>
+      <c r="C58" t="s">
+        <v>10</v>
+      </c>
+      <c r="D58" t="s">
+        <v>99</v>
+      </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
+      <c r="F58" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>136</v>
+      </c>
+      <c r="B59" t="s">
+        <v>87</v>
+      </c>
+      <c r="C59" t="s">
+        <v>29</v>
+      </c>
+      <c r="D59" t="s">
+        <v>99</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="F59" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>136</v>
+      </c>
+      <c r="B60" t="s">
+        <v>87</v>
+      </c>
+      <c r="C60" t="s">
+        <v>32</v>
+      </c>
+      <c r="D60" t="s">
+        <v>99</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>136</v>
+      </c>
+      <c r="B61" t="s">
+        <v>87</v>
+      </c>
+      <c r="C61" t="s">
+        <v>34</v>
+      </c>
+      <c r="D61" t="s">
+        <v>98</v>
+      </c>
+      <c r="E61">
+        <v>50</v>
+      </c>
+      <c r="F61" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>136</v>
+      </c>
+      <c r="B62" t="s">
+        <v>87</v>
+      </c>
+      <c r="C62" t="s">
+        <v>30</v>
+      </c>
+      <c r="D62" t="s">
+        <v>100</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+      <c r="F62" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>136</v>
+      </c>
+      <c r="B63" t="s">
+        <v>87</v>
+      </c>
+      <c r="C63" t="s">
+        <v>33</v>
+      </c>
+      <c r="D63" t="s">
+        <v>100</v>
+      </c>
+      <c r="E63">
+        <v>1</v>
+      </c>
+      <c r="F63" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>136</v>
+      </c>
+      <c r="B64" t="s">
+        <v>87</v>
+      </c>
+      <c r="C64" t="s">
+        <v>31</v>
+      </c>
+      <c r="D64" t="s">
+        <v>98</v>
+      </c>
+      <c r="E64">
+        <v>1</v>
+      </c>
+      <c r="F64" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>136</v>
+      </c>
+      <c r="B65" t="s">
+        <v>106</v>
+      </c>
+      <c r="C65" t="s">
+        <v>10</v>
+      </c>
+      <c r="D65" t="s">
+        <v>99</v>
+      </c>
+      <c r="E65">
+        <v>1</v>
+      </c>
+      <c r="F65" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>136</v>
+      </c>
+      <c r="B66" t="s">
+        <v>106</v>
+      </c>
+      <c r="C66" t="s">
+        <v>29</v>
+      </c>
+      <c r="D66" t="s">
+        <v>99</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+      <c r="F66" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>136</v>
+      </c>
+      <c r="B67" t="s">
+        <v>106</v>
+      </c>
+      <c r="C67" t="s">
+        <v>32</v>
+      </c>
+      <c r="D67" t="s">
+        <v>99</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>136</v>
+      </c>
+      <c r="B68" t="s">
+        <v>106</v>
+      </c>
+      <c r="C68" t="s">
+        <v>34</v>
+      </c>
+      <c r="D68" t="s">
+        <v>98</v>
+      </c>
+      <c r="E68">
+        <v>50</v>
+      </c>
+      <c r="F68" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>136</v>
+      </c>
+      <c r="B69" t="s">
+        <v>106</v>
+      </c>
+      <c r="C69" t="s">
+        <v>30</v>
+      </c>
+      <c r="D69" t="s">
+        <v>100</v>
+      </c>
+      <c r="E69">
+        <v>1</v>
+      </c>
+      <c r="F69" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>136</v>
+      </c>
+      <c r="B70" t="s">
+        <v>106</v>
+      </c>
+      <c r="C70" t="s">
+        <v>33</v>
+      </c>
+      <c r="D70" t="s">
+        <v>100</v>
+      </c>
+      <c r="E70">
+        <v>1</v>
+      </c>
+      <c r="F70" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>136</v>
+      </c>
+      <c r="B71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C71" t="s">
+        <v>31</v>
+      </c>
+      <c r="D71" t="s">
+        <v>98</v>
+      </c>
+      <c r="E71">
+        <v>1</v>
+      </c>
+      <c r="F71" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>136</v>
+      </c>
+      <c r="B72" t="s">
+        <v>105</v>
+      </c>
+      <c r="C72" t="s">
+        <v>10</v>
+      </c>
+      <c r="D72" t="s">
+        <v>99</v>
+      </c>
+      <c r="E72">
+        <v>1</v>
+      </c>
+      <c r="F72" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>136</v>
+      </c>
+      <c r="B73" t="s">
+        <v>105</v>
+      </c>
+      <c r="C73" t="s">
+        <v>29</v>
+      </c>
+      <c r="D73" t="s">
+        <v>99</v>
+      </c>
+      <c r="E73">
+        <v>1</v>
+      </c>
+      <c r="F73" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>136</v>
+      </c>
+      <c r="B74" t="s">
+        <v>105</v>
+      </c>
+      <c r="C74" t="s">
+        <v>32</v>
+      </c>
+      <c r="D74" t="s">
+        <v>99</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>136</v>
+      </c>
+      <c r="B75" t="s">
+        <v>105</v>
+      </c>
+      <c r="C75" t="s">
+        <v>34</v>
+      </c>
+      <c r="D75" t="s">
+        <v>98</v>
+      </c>
+      <c r="E75">
+        <v>50</v>
+      </c>
+      <c r="F75" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>136</v>
+      </c>
+      <c r="B76" t="s">
+        <v>105</v>
+      </c>
+      <c r="C76" t="s">
+        <v>30</v>
+      </c>
+      <c r="D76" t="s">
+        <v>100</v>
+      </c>
+      <c r="E76">
+        <v>1</v>
+      </c>
+      <c r="F76" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>136</v>
+      </c>
+      <c r="B77" t="s">
+        <v>105</v>
+      </c>
+      <c r="C77" t="s">
+        <v>33</v>
+      </c>
+      <c r="D77" t="s">
+        <v>100</v>
+      </c>
+      <c r="E77">
+        <v>1</v>
+      </c>
+      <c r="F77" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>136</v>
+      </c>
+      <c r="B78" t="s">
+        <v>105</v>
+      </c>
+      <c r="C78" t="s">
+        <v>31</v>
+      </c>
+      <c r="D78" t="s">
+        <v>98</v>
+      </c>
+      <c r="E78">
+        <v>1</v>
+      </c>
+      <c r="F78" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>136</v>
+      </c>
+      <c r="B79" t="s">
+        <v>107</v>
+      </c>
+      <c r="C79" t="s">
+        <v>10</v>
+      </c>
+      <c r="D79" t="s">
+        <v>99</v>
+      </c>
+      <c r="E79">
+        <v>1</v>
+      </c>
+      <c r="F79" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>136</v>
+      </c>
+      <c r="B80" t="s">
+        <v>107</v>
+      </c>
+      <c r="C80" t="s">
+        <v>29</v>
+      </c>
+      <c r="D80" t="s">
+        <v>99</v>
+      </c>
+      <c r="E80">
+        <v>1</v>
+      </c>
+      <c r="F80" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>136</v>
+      </c>
+      <c r="B81" t="s">
+        <v>107</v>
+      </c>
+      <c r="C81" t="s">
+        <v>32</v>
+      </c>
+      <c r="D81" t="s">
+        <v>99</v>
+      </c>
+      <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>136</v>
+      </c>
+      <c r="B82" t="s">
+        <v>107</v>
+      </c>
+      <c r="C82" t="s">
+        <v>34</v>
+      </c>
+      <c r="D82" t="s">
+        <v>98</v>
+      </c>
+      <c r="E82">
+        <v>50</v>
+      </c>
+      <c r="F82" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>136</v>
+      </c>
+      <c r="B83" t="s">
+        <v>107</v>
+      </c>
+      <c r="C83" t="s">
+        <v>30</v>
+      </c>
+      <c r="D83" t="s">
+        <v>100</v>
+      </c>
+      <c r="E83">
+        <v>1</v>
+      </c>
+      <c r="F83" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>136</v>
+      </c>
+      <c r="B84" t="s">
+        <v>107</v>
+      </c>
+      <c r="C84" t="s">
+        <v>33</v>
+      </c>
+      <c r="D84" t="s">
+        <v>100</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>136</v>
+      </c>
+      <c r="B85" t="s">
+        <v>107</v>
+      </c>
+      <c r="C85" t="s">
+        <v>31</v>
+      </c>
+      <c r="D85" t="s">
+        <v>98</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+      <c r="F85" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:G85" xr:uid="{7FB20890-62B7-47AF-BA68-650F053D99C5}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G260">
     <sortCondition ref="B2:B260"/>
     <sortCondition ref="A2:A260"/>
@@ -1978,7 +3021,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9375A35C-8A58-4D70-9436-2E641DE51D25}">
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G301"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -5326,13 +6369,3602 @@
         <v>96</v>
       </c>
     </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>136</v>
+      </c>
+      <c r="B146" t="s">
+        <v>71</v>
+      </c>
+      <c r="C146" t="s">
+        <v>59</v>
+      </c>
+      <c r="D146">
+        <v>0</v>
+      </c>
+      <c r="E146">
+        <v>2</v>
+      </c>
+      <c r="F146" t="s">
+        <v>43</v>
+      </c>
+      <c r="G146" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>136</v>
+      </c>
+      <c r="B147" t="s">
+        <v>71</v>
+      </c>
+      <c r="C147" t="s">
+        <v>63</v>
+      </c>
+      <c r="D147">
+        <v>1</v>
+      </c>
+      <c r="E147">
+        <v>1</v>
+      </c>
+      <c r="F147" t="s">
+        <v>43</v>
+      </c>
+      <c r="G147" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>136</v>
+      </c>
+      <c r="B148" t="s">
+        <v>71</v>
+      </c>
+      <c r="C148" t="s">
+        <v>54</v>
+      </c>
+      <c r="D148">
+        <v>2</v>
+      </c>
+      <c r="E148">
+        <v>2</v>
+      </c>
+      <c r="F148" t="s">
+        <v>43</v>
+      </c>
+      <c r="G148" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>136</v>
+      </c>
+      <c r="B149" t="s">
+        <v>71</v>
+      </c>
+      <c r="C149" t="s">
+        <v>55</v>
+      </c>
+      <c r="D149">
+        <v>3</v>
+      </c>
+      <c r="E149">
+        <v>2</v>
+      </c>
+      <c r="F149" t="s">
+        <v>43</v>
+      </c>
+      <c r="G149" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>136</v>
+      </c>
+      <c r="B150" t="s">
+        <v>71</v>
+      </c>
+      <c r="C150" t="s">
+        <v>56</v>
+      </c>
+      <c r="D150">
+        <v>4</v>
+      </c>
+      <c r="E150">
+        <v>2</v>
+      </c>
+      <c r="F150" t="s">
+        <v>43</v>
+      </c>
+      <c r="G150" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>136</v>
+      </c>
+      <c r="B151" t="s">
+        <v>71</v>
+      </c>
+      <c r="C151" t="s">
+        <v>64</v>
+      </c>
+      <c r="D151">
+        <v>5</v>
+      </c>
+      <c r="E151">
+        <v>22000</v>
+      </c>
+      <c r="F151" t="s">
+        <v>41</v>
+      </c>
+      <c r="G151" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>136</v>
+      </c>
+      <c r="B152" t="s">
+        <v>71</v>
+      </c>
+      <c r="C152" t="s">
+        <v>61</v>
+      </c>
+      <c r="D152">
+        <v>6</v>
+      </c>
+      <c r="E152">
+        <v>0</v>
+      </c>
+      <c r="F152" t="s">
+        <v>42</v>
+      </c>
+      <c r="G152" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>136</v>
+      </c>
+      <c r="B153" t="s">
+        <v>71</v>
+      </c>
+      <c r="C153" t="s">
+        <v>62</v>
+      </c>
+      <c r="D153">
+        <v>7</v>
+      </c>
+      <c r="E153">
+        <v>3</v>
+      </c>
+      <c r="F153" t="s">
+        <v>72</v>
+      </c>
+      <c r="G153" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>136</v>
+      </c>
+      <c r="B154" t="s">
+        <v>71</v>
+      </c>
+      <c r="C154" t="s">
+        <v>65</v>
+      </c>
+      <c r="D154">
+        <v>8</v>
+      </c>
+      <c r="E154">
+        <v>0.06</v>
+      </c>
+      <c r="F154" t="s">
+        <v>42</v>
+      </c>
+      <c r="G154" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>136</v>
+      </c>
+      <c r="B155" t="s">
+        <v>71</v>
+      </c>
+      <c r="C155" t="s">
+        <v>58</v>
+      </c>
+      <c r="D155">
+        <v>9</v>
+      </c>
+      <c r="E155">
+        <v>1</v>
+      </c>
+      <c r="F155" t="s">
+        <v>43</v>
+      </c>
+      <c r="G155" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>136</v>
+      </c>
+      <c r="B156" t="s">
+        <v>71</v>
+      </c>
+      <c r="C156" t="s">
+        <v>60</v>
+      </c>
+      <c r="D156">
+        <v>10</v>
+      </c>
+      <c r="E156">
+        <v>1</v>
+      </c>
+      <c r="F156" t="s">
+        <v>43</v>
+      </c>
+      <c r="G156" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>136</v>
+      </c>
+      <c r="B157" t="s">
+        <v>71</v>
+      </c>
+      <c r="C157" t="s">
+        <v>57</v>
+      </c>
+      <c r="D157">
+        <v>11</v>
+      </c>
+      <c r="E157">
+        <v>1</v>
+      </c>
+      <c r="F157" t="s">
+        <v>43</v>
+      </c>
+      <c r="G157" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>136</v>
+      </c>
+      <c r="B158" t="s">
+        <v>71</v>
+      </c>
+      <c r="C158" t="s">
+        <v>40</v>
+      </c>
+      <c r="D158">
+        <v>12</v>
+      </c>
+      <c r="E158">
+        <v>0.7</v>
+      </c>
+      <c r="F158" t="s">
+        <v>43</v>
+      </c>
+      <c r="G158" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>136</v>
+      </c>
+      <c r="B159" t="s">
+        <v>71</v>
+      </c>
+      <c r="C159" t="s">
+        <v>70</v>
+      </c>
+      <c r="D159">
+        <v>13</v>
+      </c>
+      <c r="E159">
+        <v>16</v>
+      </c>
+      <c r="F159" t="s">
+        <v>44</v>
+      </c>
+      <c r="G159" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>136</v>
+      </c>
+      <c r="B160" t="s">
+        <v>71</v>
+      </c>
+      <c r="C160" t="s">
+        <v>45</v>
+      </c>
+      <c r="D160">
+        <v>14</v>
+      </c>
+      <c r="E160">
+        <v>13</v>
+      </c>
+      <c r="F160" t="s">
+        <v>72</v>
+      </c>
+      <c r="G160" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>136</v>
+      </c>
+      <c r="B161" t="s">
+        <v>71</v>
+      </c>
+      <c r="C161" t="s">
+        <v>53</v>
+      </c>
+      <c r="D161">
+        <v>15</v>
+      </c>
+      <c r="E161">
+        <v>1</v>
+      </c>
+      <c r="F161" t="s">
+        <v>72</v>
+      </c>
+      <c r="G161" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>136</v>
+      </c>
+      <c r="B162" t="s">
+        <v>71</v>
+      </c>
+      <c r="C162" t="s">
+        <v>47</v>
+      </c>
+      <c r="D162">
+        <v>16</v>
+      </c>
+      <c r="E162">
+        <v>4</v>
+      </c>
+      <c r="F162" t="s">
+        <v>72</v>
+      </c>
+      <c r="G162" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>136</v>
+      </c>
+      <c r="B163" t="s">
+        <v>71</v>
+      </c>
+      <c r="C163" t="s">
+        <v>48</v>
+      </c>
+      <c r="D163">
+        <v>17</v>
+      </c>
+      <c r="E163">
+        <v>3</v>
+      </c>
+      <c r="F163" t="s">
+        <v>72</v>
+      </c>
+      <c r="G163" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>136</v>
+      </c>
+      <c r="B164" t="s">
+        <v>71</v>
+      </c>
+      <c r="C164" t="s">
+        <v>49</v>
+      </c>
+      <c r="D164">
+        <v>18</v>
+      </c>
+      <c r="E164">
+        <v>5</v>
+      </c>
+      <c r="F164" t="s">
+        <v>72</v>
+      </c>
+      <c r="G164" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>136</v>
+      </c>
+      <c r="B165" t="s">
+        <v>71</v>
+      </c>
+      <c r="C165" t="s">
+        <v>68</v>
+      </c>
+      <c r="D165">
+        <v>19</v>
+      </c>
+      <c r="E165">
+        <v>250000000</v>
+      </c>
+      <c r="F165" t="s">
+        <v>73</v>
+      </c>
+      <c r="G165" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B166" t="s">
+        <v>71</v>
+      </c>
+      <c r="C166" t="s">
+        <v>69</v>
+      </c>
+      <c r="D166">
+        <v>20</v>
+      </c>
+      <c r="E166">
+        <v>150000000</v>
+      </c>
+      <c r="F166" t="s">
+        <v>73</v>
+      </c>
+      <c r="G166" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>136</v>
+      </c>
+      <c r="B167" t="s">
+        <v>71</v>
+      </c>
+      <c r="C167" t="s">
+        <v>89</v>
+      </c>
+      <c r="D167">
+        <v>21</v>
+      </c>
+      <c r="E167">
+        <v>13</v>
+      </c>
+      <c r="F167" t="s">
+        <v>91</v>
+      </c>
+      <c r="G167" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>136</v>
+      </c>
+      <c r="B168" t="s">
+        <v>71</v>
+      </c>
+      <c r="C168" t="s">
+        <v>90</v>
+      </c>
+      <c r="D168">
+        <v>22</v>
+      </c>
+      <c r="E168">
+        <v>179</v>
+      </c>
+      <c r="F168" t="s">
+        <v>92</v>
+      </c>
+      <c r="G168" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>136</v>
+      </c>
+      <c r="B169" t="s">
+        <v>71</v>
+      </c>
+      <c r="C169" t="s">
+        <v>95</v>
+      </c>
+      <c r="D169">
+        <v>23</v>
+      </c>
+      <c r="E169">
+        <v>1</v>
+      </c>
+      <c r="F169" t="s">
+        <v>91</v>
+      </c>
+      <c r="G169" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>136</v>
+      </c>
+      <c r="B170" t="s">
+        <v>88</v>
+      </c>
+      <c r="C170" t="s">
+        <v>59</v>
+      </c>
+      <c r="D170">
+        <v>0</v>
+      </c>
+      <c r="E170">
+        <v>0</v>
+      </c>
+      <c r="F170" t="s">
+        <v>43</v>
+      </c>
+      <c r="G170" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>136</v>
+      </c>
+      <c r="B171" t="s">
+        <v>88</v>
+      </c>
+      <c r="C171" t="s">
+        <v>63</v>
+      </c>
+      <c r="D171">
+        <v>1</v>
+      </c>
+      <c r="E171">
+        <v>0</v>
+      </c>
+      <c r="F171" t="s">
+        <v>43</v>
+      </c>
+      <c r="G171" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>136</v>
+      </c>
+      <c r="B172" t="s">
+        <v>88</v>
+      </c>
+      <c r="C172" t="s">
+        <v>54</v>
+      </c>
+      <c r="D172">
+        <v>2</v>
+      </c>
+      <c r="E172">
+        <v>0</v>
+      </c>
+      <c r="F172" t="s">
+        <v>43</v>
+      </c>
+      <c r="G172" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>136</v>
+      </c>
+      <c r="B173" t="s">
+        <v>88</v>
+      </c>
+      <c r="C173" t="s">
+        <v>55</v>
+      </c>
+      <c r="D173">
+        <v>3</v>
+      </c>
+      <c r="E173">
+        <v>0</v>
+      </c>
+      <c r="F173" t="s">
+        <v>43</v>
+      </c>
+      <c r="G173" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>136</v>
+      </c>
+      <c r="B174" t="s">
+        <v>88</v>
+      </c>
+      <c r="C174" t="s">
+        <v>56</v>
+      </c>
+      <c r="D174">
+        <v>4</v>
+      </c>
+      <c r="E174">
+        <v>0</v>
+      </c>
+      <c r="F174" t="s">
+        <v>43</v>
+      </c>
+      <c r="G174" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>136</v>
+      </c>
+      <c r="B175" t="s">
+        <v>88</v>
+      </c>
+      <c r="C175" t="s">
+        <v>64</v>
+      </c>
+      <c r="D175">
+        <v>5</v>
+      </c>
+      <c r="E175">
+        <v>1000000</v>
+      </c>
+      <c r="F175" t="s">
+        <v>41</v>
+      </c>
+      <c r="G175" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>136</v>
+      </c>
+      <c r="B176" t="s">
+        <v>88</v>
+      </c>
+      <c r="C176" t="s">
+        <v>61</v>
+      </c>
+      <c r="D176">
+        <v>6</v>
+      </c>
+      <c r="E176">
+        <v>0</v>
+      </c>
+      <c r="F176" t="s">
+        <v>42</v>
+      </c>
+      <c r="G176" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>136</v>
+      </c>
+      <c r="B177" t="s">
+        <v>88</v>
+      </c>
+      <c r="C177" t="s">
+        <v>62</v>
+      </c>
+      <c r="D177">
+        <v>7</v>
+      </c>
+      <c r="E177">
+        <v>13</v>
+      </c>
+      <c r="F177" t="s">
+        <v>72</v>
+      </c>
+      <c r="G177" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>136</v>
+      </c>
+      <c r="B178" t="s">
+        <v>88</v>
+      </c>
+      <c r="C178" t="s">
+        <v>65</v>
+      </c>
+      <c r="D178">
+        <v>8</v>
+      </c>
+      <c r="E178">
+        <v>0.15</v>
+      </c>
+      <c r="F178" t="s">
+        <v>42</v>
+      </c>
+      <c r="G178" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>136</v>
+      </c>
+      <c r="B179" t="s">
+        <v>88</v>
+      </c>
+      <c r="C179" t="s">
+        <v>58</v>
+      </c>
+      <c r="D179">
+        <v>9</v>
+      </c>
+      <c r="E179">
+        <v>0</v>
+      </c>
+      <c r="F179" t="s">
+        <v>43</v>
+      </c>
+      <c r="G179" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>136</v>
+      </c>
+      <c r="B180" t="s">
+        <v>88</v>
+      </c>
+      <c r="C180" t="s">
+        <v>60</v>
+      </c>
+      <c r="D180">
+        <v>10</v>
+      </c>
+      <c r="E180">
+        <v>0</v>
+      </c>
+      <c r="F180" t="s">
+        <v>43</v>
+      </c>
+      <c r="G180" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>136</v>
+      </c>
+      <c r="B181" t="s">
+        <v>88</v>
+      </c>
+      <c r="C181" t="s">
+        <v>57</v>
+      </c>
+      <c r="D181">
+        <v>11</v>
+      </c>
+      <c r="E181">
+        <v>0</v>
+      </c>
+      <c r="F181" t="s">
+        <v>43</v>
+      </c>
+      <c r="G181" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>136</v>
+      </c>
+      <c r="B182" t="s">
+        <v>88</v>
+      </c>
+      <c r="C182" t="s">
+        <v>40</v>
+      </c>
+      <c r="D182">
+        <v>12</v>
+      </c>
+      <c r="E182">
+        <v>0.7</v>
+      </c>
+      <c r="F182" t="s">
+        <v>43</v>
+      </c>
+      <c r="G182" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>136</v>
+      </c>
+      <c r="B183" t="s">
+        <v>88</v>
+      </c>
+      <c r="C183" t="s">
+        <v>70</v>
+      </c>
+      <c r="D183">
+        <v>13</v>
+      </c>
+      <c r="E183">
+        <v>24</v>
+      </c>
+      <c r="F183" t="s">
+        <v>44</v>
+      </c>
+      <c r="G183" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>136</v>
+      </c>
+      <c r="B184" t="s">
+        <v>88</v>
+      </c>
+      <c r="C184" t="s">
+        <v>45</v>
+      </c>
+      <c r="D184">
+        <v>14</v>
+      </c>
+      <c r="E184">
+        <v>13</v>
+      </c>
+      <c r="F184" t="s">
+        <v>72</v>
+      </c>
+      <c r="G184" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>136</v>
+      </c>
+      <c r="B185" t="s">
+        <v>88</v>
+      </c>
+      <c r="C185" t="s">
+        <v>53</v>
+      </c>
+      <c r="D185">
+        <v>15</v>
+      </c>
+      <c r="E185">
+        <v>1</v>
+      </c>
+      <c r="F185" t="s">
+        <v>72</v>
+      </c>
+      <c r="G185" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>136</v>
+      </c>
+      <c r="B186" t="s">
+        <v>88</v>
+      </c>
+      <c r="C186" t="s">
+        <v>47</v>
+      </c>
+      <c r="D186">
+        <v>16</v>
+      </c>
+      <c r="E186">
+        <v>13</v>
+      </c>
+      <c r="F186" t="s">
+        <v>72</v>
+      </c>
+      <c r="G186" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>136</v>
+      </c>
+      <c r="B187" t="s">
+        <v>88</v>
+      </c>
+      <c r="C187" t="s">
+        <v>48</v>
+      </c>
+      <c r="D187">
+        <v>17</v>
+      </c>
+      <c r="E187">
+        <v>13</v>
+      </c>
+      <c r="F187" t="s">
+        <v>72</v>
+      </c>
+      <c r="G187" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>136</v>
+      </c>
+      <c r="B188" t="s">
+        <v>88</v>
+      </c>
+      <c r="C188" t="s">
+        <v>49</v>
+      </c>
+      <c r="D188">
+        <v>18</v>
+      </c>
+      <c r="E188">
+        <v>13</v>
+      </c>
+      <c r="F188" t="s">
+        <v>72</v>
+      </c>
+      <c r="G188" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>136</v>
+      </c>
+      <c r="B189" t="s">
+        <v>88</v>
+      </c>
+      <c r="C189" t="s">
+        <v>68</v>
+      </c>
+      <c r="D189">
+        <v>19</v>
+      </c>
+      <c r="E189">
+        <v>250000000</v>
+      </c>
+      <c r="F189" t="s">
+        <v>73</v>
+      </c>
+      <c r="G189" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>136</v>
+      </c>
+      <c r="B190" t="s">
+        <v>88</v>
+      </c>
+      <c r="C190" t="s">
+        <v>69</v>
+      </c>
+      <c r="D190">
+        <v>20</v>
+      </c>
+      <c r="E190">
+        <v>150000000</v>
+      </c>
+      <c r="F190" t="s">
+        <v>73</v>
+      </c>
+      <c r="G190" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>136</v>
+      </c>
+      <c r="B191" t="s">
+        <v>88</v>
+      </c>
+      <c r="C191" t="s">
+        <v>89</v>
+      </c>
+      <c r="D191">
+        <v>21</v>
+      </c>
+      <c r="E191">
+        <v>13</v>
+      </c>
+      <c r="F191" t="s">
+        <v>91</v>
+      </c>
+      <c r="G191" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>136</v>
+      </c>
+      <c r="B192" t="s">
+        <v>88</v>
+      </c>
+      <c r="C192" t="s">
+        <v>90</v>
+      </c>
+      <c r="D192">
+        <v>22</v>
+      </c>
+      <c r="E192">
+        <v>179</v>
+      </c>
+      <c r="F192" t="s">
+        <v>92</v>
+      </c>
+      <c r="G192" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>136</v>
+      </c>
+      <c r="B193" t="s">
+        <v>88</v>
+      </c>
+      <c r="C193" t="s">
+        <v>95</v>
+      </c>
+      <c r="D193">
+        <v>23</v>
+      </c>
+      <c r="E193">
+        <v>1</v>
+      </c>
+      <c r="F193" t="s">
+        <v>91</v>
+      </c>
+      <c r="G193" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>136</v>
+      </c>
+      <c r="B194" t="s">
+        <v>87</v>
+      </c>
+      <c r="C194" t="s">
+        <v>59</v>
+      </c>
+      <c r="D194">
+        <v>0</v>
+      </c>
+      <c r="E194">
+        <v>2</v>
+      </c>
+      <c r="F194" t="s">
+        <v>43</v>
+      </c>
+      <c r="G194" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>136</v>
+      </c>
+      <c r="B195" t="s">
+        <v>87</v>
+      </c>
+      <c r="C195" t="s">
+        <v>63</v>
+      </c>
+      <c r="D195">
+        <v>1</v>
+      </c>
+      <c r="E195">
+        <v>1</v>
+      </c>
+      <c r="F195" t="s">
+        <v>43</v>
+      </c>
+      <c r="G195" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>136</v>
+      </c>
+      <c r="B196" t="s">
+        <v>87</v>
+      </c>
+      <c r="C196" t="s">
+        <v>54</v>
+      </c>
+      <c r="D196">
+        <v>2</v>
+      </c>
+      <c r="E196">
+        <v>2</v>
+      </c>
+      <c r="F196" t="s">
+        <v>43</v>
+      </c>
+      <c r="G196" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>136</v>
+      </c>
+      <c r="B197" t="s">
+        <v>87</v>
+      </c>
+      <c r="C197" t="s">
+        <v>55</v>
+      </c>
+      <c r="D197">
+        <v>3</v>
+      </c>
+      <c r="E197">
+        <v>2</v>
+      </c>
+      <c r="F197" t="s">
+        <v>43</v>
+      </c>
+      <c r="G197" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>136</v>
+      </c>
+      <c r="B198" t="s">
+        <v>87</v>
+      </c>
+      <c r="C198" t="s">
+        <v>56</v>
+      </c>
+      <c r="D198">
+        <v>4</v>
+      </c>
+      <c r="E198">
+        <v>2</v>
+      </c>
+      <c r="F198" t="s">
+        <v>43</v>
+      </c>
+      <c r="G198" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>136</v>
+      </c>
+      <c r="B199" t="s">
+        <v>87</v>
+      </c>
+      <c r="C199" t="s">
+        <v>64</v>
+      </c>
+      <c r="D199">
+        <v>5</v>
+      </c>
+      <c r="E199">
+        <v>22000</v>
+      </c>
+      <c r="F199" t="s">
+        <v>41</v>
+      </c>
+      <c r="G199" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>136</v>
+      </c>
+      <c r="B200" t="s">
+        <v>87</v>
+      </c>
+      <c r="C200" t="s">
+        <v>61</v>
+      </c>
+      <c r="D200">
+        <v>6</v>
+      </c>
+      <c r="E200">
+        <v>0.4</v>
+      </c>
+      <c r="F200" t="s">
+        <v>42</v>
+      </c>
+      <c r="G200" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>136</v>
+      </c>
+      <c r="B201" t="s">
+        <v>87</v>
+      </c>
+      <c r="C201" t="s">
+        <v>62</v>
+      </c>
+      <c r="D201">
+        <v>7</v>
+      </c>
+      <c r="E201">
+        <v>3</v>
+      </c>
+      <c r="F201" t="s">
+        <v>72</v>
+      </c>
+      <c r="G201" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>136</v>
+      </c>
+      <c r="B202" t="s">
+        <v>87</v>
+      </c>
+      <c r="C202" t="s">
+        <v>65</v>
+      </c>
+      <c r="D202">
+        <v>8</v>
+      </c>
+      <c r="E202">
+        <v>0.06</v>
+      </c>
+      <c r="F202" t="s">
+        <v>42</v>
+      </c>
+      <c r="G202" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>136</v>
+      </c>
+      <c r="B203" t="s">
+        <v>87</v>
+      </c>
+      <c r="C203" t="s">
+        <v>58</v>
+      </c>
+      <c r="D203">
+        <v>9</v>
+      </c>
+      <c r="E203">
+        <v>1</v>
+      </c>
+      <c r="F203" t="s">
+        <v>43</v>
+      </c>
+      <c r="G203" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>136</v>
+      </c>
+      <c r="B204" t="s">
+        <v>87</v>
+      </c>
+      <c r="C204" t="s">
+        <v>60</v>
+      </c>
+      <c r="D204">
+        <v>10</v>
+      </c>
+      <c r="E204">
+        <v>1</v>
+      </c>
+      <c r="F204" t="s">
+        <v>43</v>
+      </c>
+      <c r="G204" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>136</v>
+      </c>
+      <c r="B205" t="s">
+        <v>87</v>
+      </c>
+      <c r="C205" t="s">
+        <v>57</v>
+      </c>
+      <c r="D205">
+        <v>11</v>
+      </c>
+      <c r="E205">
+        <v>1</v>
+      </c>
+      <c r="F205" t="s">
+        <v>43</v>
+      </c>
+      <c r="G205" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>136</v>
+      </c>
+      <c r="B206" t="s">
+        <v>87</v>
+      </c>
+      <c r="C206" t="s">
+        <v>40</v>
+      </c>
+      <c r="D206">
+        <v>12</v>
+      </c>
+      <c r="E206">
+        <v>1</v>
+      </c>
+      <c r="F206" t="s">
+        <v>43</v>
+      </c>
+      <c r="G206" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>136</v>
+      </c>
+      <c r="B207" t="s">
+        <v>87</v>
+      </c>
+      <c r="C207" t="s">
+        <v>70</v>
+      </c>
+      <c r="D207">
+        <v>13</v>
+      </c>
+      <c r="E207">
+        <v>3</v>
+      </c>
+      <c r="F207" t="s">
+        <v>44</v>
+      </c>
+      <c r="G207" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>136</v>
+      </c>
+      <c r="B208" t="s">
+        <v>87</v>
+      </c>
+      <c r="C208" t="s">
+        <v>45</v>
+      </c>
+      <c r="D208">
+        <v>14</v>
+      </c>
+      <c r="E208">
+        <v>13</v>
+      </c>
+      <c r="F208" t="s">
+        <v>72</v>
+      </c>
+      <c r="G208" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>136</v>
+      </c>
+      <c r="B209" t="s">
+        <v>87</v>
+      </c>
+      <c r="C209" t="s">
+        <v>53</v>
+      </c>
+      <c r="D209">
+        <v>15</v>
+      </c>
+      <c r="E209">
+        <v>1</v>
+      </c>
+      <c r="F209" t="s">
+        <v>72</v>
+      </c>
+      <c r="G209" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>136</v>
+      </c>
+      <c r="B210" t="s">
+        <v>87</v>
+      </c>
+      <c r="C210" t="s">
+        <v>47</v>
+      </c>
+      <c r="D210">
+        <v>16</v>
+      </c>
+      <c r="E210">
+        <v>1</v>
+      </c>
+      <c r="F210" t="s">
+        <v>72</v>
+      </c>
+      <c r="G210" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>136</v>
+      </c>
+      <c r="B211" t="s">
+        <v>87</v>
+      </c>
+      <c r="C211" t="s">
+        <v>48</v>
+      </c>
+      <c r="D211">
+        <v>17</v>
+      </c>
+      <c r="E211">
+        <v>1</v>
+      </c>
+      <c r="F211" t="s">
+        <v>72</v>
+      </c>
+      <c r="G211" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>136</v>
+      </c>
+      <c r="B212" t="s">
+        <v>87</v>
+      </c>
+      <c r="C212" t="s">
+        <v>49</v>
+      </c>
+      <c r="D212">
+        <v>18</v>
+      </c>
+      <c r="E212">
+        <v>1</v>
+      </c>
+      <c r="F212" t="s">
+        <v>72</v>
+      </c>
+      <c r="G212" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>136</v>
+      </c>
+      <c r="B213" t="s">
+        <v>87</v>
+      </c>
+      <c r="C213" t="s">
+        <v>68</v>
+      </c>
+      <c r="D213">
+        <v>19</v>
+      </c>
+      <c r="E213">
+        <v>250000000</v>
+      </c>
+      <c r="F213" t="s">
+        <v>73</v>
+      </c>
+      <c r="G213" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>136</v>
+      </c>
+      <c r="B214" t="s">
+        <v>87</v>
+      </c>
+      <c r="C214" t="s">
+        <v>69</v>
+      </c>
+      <c r="D214">
+        <v>20</v>
+      </c>
+      <c r="E214">
+        <v>150000000</v>
+      </c>
+      <c r="F214" t="s">
+        <v>73</v>
+      </c>
+      <c r="G214" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>136</v>
+      </c>
+      <c r="B215" t="s">
+        <v>87</v>
+      </c>
+      <c r="C215" t="s">
+        <v>89</v>
+      </c>
+      <c r="D215">
+        <v>21</v>
+      </c>
+      <c r="E215">
+        <v>13</v>
+      </c>
+      <c r="F215" t="s">
+        <v>91</v>
+      </c>
+      <c r="G215" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>136</v>
+      </c>
+      <c r="B216" t="s">
+        <v>87</v>
+      </c>
+      <c r="C216" t="s">
+        <v>90</v>
+      </c>
+      <c r="D216">
+        <v>22</v>
+      </c>
+      <c r="E216">
+        <v>179</v>
+      </c>
+      <c r="F216" t="s">
+        <v>92</v>
+      </c>
+      <c r="G216" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>136</v>
+      </c>
+      <c r="B217" t="s">
+        <v>87</v>
+      </c>
+      <c r="C217" t="s">
+        <v>95</v>
+      </c>
+      <c r="D217">
+        <v>23</v>
+      </c>
+      <c r="E217">
+        <v>1</v>
+      </c>
+      <c r="F217" t="s">
+        <v>91</v>
+      </c>
+      <c r="G217" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>136</v>
+      </c>
+      <c r="B218" t="s">
+        <v>106</v>
+      </c>
+      <c r="C218" t="s">
+        <v>59</v>
+      </c>
+      <c r="D218">
+        <v>0</v>
+      </c>
+      <c r="E218">
+        <v>2</v>
+      </c>
+      <c r="F218" t="s">
+        <v>43</v>
+      </c>
+      <c r="G218" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>136</v>
+      </c>
+      <c r="B219" t="s">
+        <v>106</v>
+      </c>
+      <c r="C219" t="s">
+        <v>63</v>
+      </c>
+      <c r="D219">
+        <v>1</v>
+      </c>
+      <c r="E219">
+        <v>1</v>
+      </c>
+      <c r="F219" t="s">
+        <v>43</v>
+      </c>
+      <c r="G219" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>136</v>
+      </c>
+      <c r="B220" t="s">
+        <v>106</v>
+      </c>
+      <c r="C220" t="s">
+        <v>54</v>
+      </c>
+      <c r="D220">
+        <v>2</v>
+      </c>
+      <c r="E220">
+        <v>2</v>
+      </c>
+      <c r="F220" t="s">
+        <v>43</v>
+      </c>
+      <c r="G220" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>136</v>
+      </c>
+      <c r="B221" t="s">
+        <v>106</v>
+      </c>
+      <c r="C221" t="s">
+        <v>55</v>
+      </c>
+      <c r="D221">
+        <v>3</v>
+      </c>
+      <c r="E221">
+        <v>2</v>
+      </c>
+      <c r="F221" t="s">
+        <v>43</v>
+      </c>
+      <c r="G221" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>136</v>
+      </c>
+      <c r="B222" t="s">
+        <v>106</v>
+      </c>
+      <c r="C222" t="s">
+        <v>56</v>
+      </c>
+      <c r="D222">
+        <v>4</v>
+      </c>
+      <c r="E222">
+        <v>2</v>
+      </c>
+      <c r="F222" t="s">
+        <v>43</v>
+      </c>
+      <c r="G222" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>136</v>
+      </c>
+      <c r="B223" t="s">
+        <v>106</v>
+      </c>
+      <c r="C223" t="s">
+        <v>64</v>
+      </c>
+      <c r="D223">
+        <v>5</v>
+      </c>
+      <c r="E223">
+        <v>22000</v>
+      </c>
+      <c r="F223" t="s">
+        <v>41</v>
+      </c>
+      <c r="G223" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>136</v>
+      </c>
+      <c r="B224" t="s">
+        <v>106</v>
+      </c>
+      <c r="C224" t="s">
+        <v>61</v>
+      </c>
+      <c r="D224">
+        <v>6</v>
+      </c>
+      <c r="E224">
+        <v>0.4</v>
+      </c>
+      <c r="F224" t="s">
+        <v>42</v>
+      </c>
+      <c r="G224" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>136</v>
+      </c>
+      <c r="B225" t="s">
+        <v>106</v>
+      </c>
+      <c r="C225" t="s">
+        <v>62</v>
+      </c>
+      <c r="D225">
+        <v>7</v>
+      </c>
+      <c r="E225">
+        <v>3</v>
+      </c>
+      <c r="F225" t="s">
+        <v>72</v>
+      </c>
+      <c r="G225" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>136</v>
+      </c>
+      <c r="B226" t="s">
+        <v>106</v>
+      </c>
+      <c r="C226" t="s">
+        <v>65</v>
+      </c>
+      <c r="D226">
+        <v>8</v>
+      </c>
+      <c r="E226">
+        <v>0.06</v>
+      </c>
+      <c r="F226" t="s">
+        <v>42</v>
+      </c>
+      <c r="G226" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>136</v>
+      </c>
+      <c r="B227" t="s">
+        <v>106</v>
+      </c>
+      <c r="C227" t="s">
+        <v>58</v>
+      </c>
+      <c r="D227">
+        <v>9</v>
+      </c>
+      <c r="E227">
+        <v>1</v>
+      </c>
+      <c r="F227" t="s">
+        <v>43</v>
+      </c>
+      <c r="G227" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>136</v>
+      </c>
+      <c r="B228" t="s">
+        <v>106</v>
+      </c>
+      <c r="C228" t="s">
+        <v>60</v>
+      </c>
+      <c r="D228">
+        <v>10</v>
+      </c>
+      <c r="E228">
+        <v>1</v>
+      </c>
+      <c r="F228" t="s">
+        <v>43</v>
+      </c>
+      <c r="G228" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>136</v>
+      </c>
+      <c r="B229" t="s">
+        <v>106</v>
+      </c>
+      <c r="C229" t="s">
+        <v>57</v>
+      </c>
+      <c r="D229">
+        <v>11</v>
+      </c>
+      <c r="E229">
+        <v>1</v>
+      </c>
+      <c r="F229" t="s">
+        <v>43</v>
+      </c>
+      <c r="G229" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>136</v>
+      </c>
+      <c r="B230" t="s">
+        <v>106</v>
+      </c>
+      <c r="C230" t="s">
+        <v>40</v>
+      </c>
+      <c r="D230">
+        <v>12</v>
+      </c>
+      <c r="E230">
+        <v>1</v>
+      </c>
+      <c r="F230" t="s">
+        <v>43</v>
+      </c>
+      <c r="G230" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>136</v>
+      </c>
+      <c r="B231" t="s">
+        <v>106</v>
+      </c>
+      <c r="C231" t="s">
+        <v>70</v>
+      </c>
+      <c r="D231">
+        <v>13</v>
+      </c>
+      <c r="E231">
+        <v>3</v>
+      </c>
+      <c r="F231" t="s">
+        <v>44</v>
+      </c>
+      <c r="G231" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>136</v>
+      </c>
+      <c r="B232" t="s">
+        <v>106</v>
+      </c>
+      <c r="C232" t="s">
+        <v>45</v>
+      </c>
+      <c r="D232">
+        <v>14</v>
+      </c>
+      <c r="E232">
+        <v>13</v>
+      </c>
+      <c r="F232" t="s">
+        <v>72</v>
+      </c>
+      <c r="G232" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>136</v>
+      </c>
+      <c r="B233" t="s">
+        <v>106</v>
+      </c>
+      <c r="C233" t="s">
+        <v>53</v>
+      </c>
+      <c r="D233">
+        <v>15</v>
+      </c>
+      <c r="E233">
+        <v>13</v>
+      </c>
+      <c r="F233" t="s">
+        <v>72</v>
+      </c>
+      <c r="G233" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>136</v>
+      </c>
+      <c r="B234" t="s">
+        <v>106</v>
+      </c>
+      <c r="C234" t="s">
+        <v>47</v>
+      </c>
+      <c r="D234">
+        <v>16</v>
+      </c>
+      <c r="E234">
+        <v>1</v>
+      </c>
+      <c r="F234" t="s">
+        <v>72</v>
+      </c>
+      <c r="G234" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>136</v>
+      </c>
+      <c r="B235" t="s">
+        <v>106</v>
+      </c>
+      <c r="C235" t="s">
+        <v>48</v>
+      </c>
+      <c r="D235">
+        <v>17</v>
+      </c>
+      <c r="E235">
+        <v>1</v>
+      </c>
+      <c r="F235" t="s">
+        <v>72</v>
+      </c>
+      <c r="G235" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>136</v>
+      </c>
+      <c r="B236" t="s">
+        <v>106</v>
+      </c>
+      <c r="C236" t="s">
+        <v>49</v>
+      </c>
+      <c r="D236">
+        <v>18</v>
+      </c>
+      <c r="E236">
+        <v>1</v>
+      </c>
+      <c r="F236" t="s">
+        <v>72</v>
+      </c>
+      <c r="G236" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>136</v>
+      </c>
+      <c r="B237" t="s">
+        <v>106</v>
+      </c>
+      <c r="C237" t="s">
+        <v>68</v>
+      </c>
+      <c r="D237">
+        <v>19</v>
+      </c>
+      <c r="E237">
+        <v>250000000</v>
+      </c>
+      <c r="F237" t="s">
+        <v>73</v>
+      </c>
+      <c r="G237" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>136</v>
+      </c>
+      <c r="B238" t="s">
+        <v>106</v>
+      </c>
+      <c r="C238" t="s">
+        <v>69</v>
+      </c>
+      <c r="D238">
+        <v>20</v>
+      </c>
+      <c r="E238">
+        <v>150000000</v>
+      </c>
+      <c r="F238" t="s">
+        <v>73</v>
+      </c>
+      <c r="G238" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>136</v>
+      </c>
+      <c r="B239" t="s">
+        <v>106</v>
+      </c>
+      <c r="C239" t="s">
+        <v>89</v>
+      </c>
+      <c r="D239">
+        <v>21</v>
+      </c>
+      <c r="E239">
+        <v>13</v>
+      </c>
+      <c r="F239" t="s">
+        <v>91</v>
+      </c>
+      <c r="G239" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>136</v>
+      </c>
+      <c r="B240" t="s">
+        <v>106</v>
+      </c>
+      <c r="C240" t="s">
+        <v>90</v>
+      </c>
+      <c r="D240">
+        <v>22</v>
+      </c>
+      <c r="E240">
+        <v>179</v>
+      </c>
+      <c r="F240" t="s">
+        <v>92</v>
+      </c>
+      <c r="G240" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>136</v>
+      </c>
+      <c r="B241" t="s">
+        <v>106</v>
+      </c>
+      <c r="C241" t="s">
+        <v>95</v>
+      </c>
+      <c r="D241">
+        <v>23</v>
+      </c>
+      <c r="E241">
+        <v>1</v>
+      </c>
+      <c r="F241" t="s">
+        <v>91</v>
+      </c>
+      <c r="G241" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>136</v>
+      </c>
+      <c r="B242" t="s">
+        <v>105</v>
+      </c>
+      <c r="C242" t="s">
+        <v>59</v>
+      </c>
+      <c r="D242">
+        <v>0</v>
+      </c>
+      <c r="E242">
+        <v>0</v>
+      </c>
+      <c r="F242" t="s">
+        <v>43</v>
+      </c>
+      <c r="G242" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>136</v>
+      </c>
+      <c r="B243" t="s">
+        <v>105</v>
+      </c>
+      <c r="C243" t="s">
+        <v>63</v>
+      </c>
+      <c r="D243">
+        <v>1</v>
+      </c>
+      <c r="E243">
+        <v>0</v>
+      </c>
+      <c r="F243" t="s">
+        <v>43</v>
+      </c>
+      <c r="G243" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>136</v>
+      </c>
+      <c r="B244" t="s">
+        <v>105</v>
+      </c>
+      <c r="C244" t="s">
+        <v>54</v>
+      </c>
+      <c r="D244">
+        <v>2</v>
+      </c>
+      <c r="E244">
+        <v>0</v>
+      </c>
+      <c r="F244" t="s">
+        <v>43</v>
+      </c>
+      <c r="G244" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>136</v>
+      </c>
+      <c r="B245" t="s">
+        <v>105</v>
+      </c>
+      <c r="C245" t="s">
+        <v>55</v>
+      </c>
+      <c r="D245">
+        <v>3</v>
+      </c>
+      <c r="E245">
+        <v>0</v>
+      </c>
+      <c r="F245" t="s">
+        <v>43</v>
+      </c>
+      <c r="G245" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>136</v>
+      </c>
+      <c r="B246" t="s">
+        <v>105</v>
+      </c>
+      <c r="C246" t="s">
+        <v>56</v>
+      </c>
+      <c r="D246">
+        <v>4</v>
+      </c>
+      <c r="E246">
+        <v>0</v>
+      </c>
+      <c r="F246" t="s">
+        <v>43</v>
+      </c>
+      <c r="G246" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>136</v>
+      </c>
+      <c r="B247" t="s">
+        <v>105</v>
+      </c>
+      <c r="C247" t="s">
+        <v>64</v>
+      </c>
+      <c r="D247">
+        <v>5</v>
+      </c>
+      <c r="E247">
+        <v>1000000</v>
+      </c>
+      <c r="F247" t="s">
+        <v>41</v>
+      </c>
+      <c r="G247" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>136</v>
+      </c>
+      <c r="B248" t="s">
+        <v>105</v>
+      </c>
+      <c r="C248" t="s">
+        <v>61</v>
+      </c>
+      <c r="D248">
+        <v>6</v>
+      </c>
+      <c r="E248">
+        <v>0</v>
+      </c>
+      <c r="F248" t="s">
+        <v>42</v>
+      </c>
+      <c r="G248" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>136</v>
+      </c>
+      <c r="B249" t="s">
+        <v>105</v>
+      </c>
+      <c r="C249" t="s">
+        <v>62</v>
+      </c>
+      <c r="D249">
+        <v>7</v>
+      </c>
+      <c r="E249">
+        <v>13</v>
+      </c>
+      <c r="F249" t="s">
+        <v>72</v>
+      </c>
+      <c r="G249" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>136</v>
+      </c>
+      <c r="B250" t="s">
+        <v>105</v>
+      </c>
+      <c r="C250" t="s">
+        <v>65</v>
+      </c>
+      <c r="D250">
+        <v>8</v>
+      </c>
+      <c r="E250">
+        <v>0.15</v>
+      </c>
+      <c r="F250" t="s">
+        <v>42</v>
+      </c>
+      <c r="G250" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>136</v>
+      </c>
+      <c r="B251" t="s">
+        <v>105</v>
+      </c>
+      <c r="C251" t="s">
+        <v>58</v>
+      </c>
+      <c r="D251">
+        <v>9</v>
+      </c>
+      <c r="E251">
+        <v>0</v>
+      </c>
+      <c r="F251" t="s">
+        <v>43</v>
+      </c>
+      <c r="G251" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>136</v>
+      </c>
+      <c r="B252" t="s">
+        <v>105</v>
+      </c>
+      <c r="C252" t="s">
+        <v>60</v>
+      </c>
+      <c r="D252">
+        <v>10</v>
+      </c>
+      <c r="E252">
+        <v>0</v>
+      </c>
+      <c r="F252" t="s">
+        <v>43</v>
+      </c>
+      <c r="G252" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>136</v>
+      </c>
+      <c r="B253" t="s">
+        <v>105</v>
+      </c>
+      <c r="C253" t="s">
+        <v>57</v>
+      </c>
+      <c r="D253">
+        <v>11</v>
+      </c>
+      <c r="E253">
+        <v>0</v>
+      </c>
+      <c r="F253" t="s">
+        <v>43</v>
+      </c>
+      <c r="G253" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>136</v>
+      </c>
+      <c r="B254" t="s">
+        <v>105</v>
+      </c>
+      <c r="C254" t="s">
+        <v>40</v>
+      </c>
+      <c r="D254">
+        <v>12</v>
+      </c>
+      <c r="E254">
+        <v>0.7</v>
+      </c>
+      <c r="F254" t="s">
+        <v>43</v>
+      </c>
+      <c r="G254" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
+        <v>136</v>
+      </c>
+      <c r="B255" t="s">
+        <v>105</v>
+      </c>
+      <c r="C255" t="s">
+        <v>70</v>
+      </c>
+      <c r="D255">
+        <v>13</v>
+      </c>
+      <c r="E255">
+        <v>24</v>
+      </c>
+      <c r="F255" t="s">
+        <v>44</v>
+      </c>
+      <c r="G255" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
+        <v>136</v>
+      </c>
+      <c r="B256" t="s">
+        <v>105</v>
+      </c>
+      <c r="C256" t="s">
+        <v>45</v>
+      </c>
+      <c r="D256">
+        <v>14</v>
+      </c>
+      <c r="E256">
+        <v>13</v>
+      </c>
+      <c r="F256" t="s">
+        <v>72</v>
+      </c>
+      <c r="G256" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
+        <v>136</v>
+      </c>
+      <c r="B257" t="s">
+        <v>105</v>
+      </c>
+      <c r="C257" t="s">
+        <v>53</v>
+      </c>
+      <c r="D257">
+        <v>15</v>
+      </c>
+      <c r="E257">
+        <v>13</v>
+      </c>
+      <c r="F257" t="s">
+        <v>72</v>
+      </c>
+      <c r="G257" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A258" t="s">
+        <v>136</v>
+      </c>
+      <c r="B258" t="s">
+        <v>105</v>
+      </c>
+      <c r="C258" t="s">
+        <v>47</v>
+      </c>
+      <c r="D258">
+        <v>16</v>
+      </c>
+      <c r="E258">
+        <v>13</v>
+      </c>
+      <c r="F258" t="s">
+        <v>72</v>
+      </c>
+      <c r="G258" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A259" t="s">
+        <v>136</v>
+      </c>
+      <c r="B259" t="s">
+        <v>105</v>
+      </c>
+      <c r="C259" t="s">
+        <v>48</v>
+      </c>
+      <c r="D259">
+        <v>17</v>
+      </c>
+      <c r="E259">
+        <v>13</v>
+      </c>
+      <c r="F259" t="s">
+        <v>72</v>
+      </c>
+      <c r="G259" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A260" t="s">
+        <v>136</v>
+      </c>
+      <c r="B260" t="s">
+        <v>105</v>
+      </c>
+      <c r="C260" t="s">
+        <v>49</v>
+      </c>
+      <c r="D260">
+        <v>18</v>
+      </c>
+      <c r="E260">
+        <v>13</v>
+      </c>
+      <c r="F260" t="s">
+        <v>72</v>
+      </c>
+      <c r="G260" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A261" t="s">
+        <v>136</v>
+      </c>
+      <c r="B261" t="s">
+        <v>105</v>
+      </c>
+      <c r="C261" t="s">
+        <v>68</v>
+      </c>
+      <c r="D261">
+        <v>19</v>
+      </c>
+      <c r="E261">
+        <v>250000000</v>
+      </c>
+      <c r="F261" t="s">
+        <v>73</v>
+      </c>
+      <c r="G261" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A262" t="s">
+        <v>136</v>
+      </c>
+      <c r="B262" t="s">
+        <v>105</v>
+      </c>
+      <c r="C262" t="s">
+        <v>69</v>
+      </c>
+      <c r="D262">
+        <v>20</v>
+      </c>
+      <c r="E262">
+        <v>150000000</v>
+      </c>
+      <c r="F262" t="s">
+        <v>73</v>
+      </c>
+      <c r="G262" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A263" t="s">
+        <v>136</v>
+      </c>
+      <c r="B263" t="s">
+        <v>105</v>
+      </c>
+      <c r="C263" t="s">
+        <v>89</v>
+      </c>
+      <c r="D263">
+        <v>21</v>
+      </c>
+      <c r="E263">
+        <v>13</v>
+      </c>
+      <c r="F263" t="s">
+        <v>91</v>
+      </c>
+      <c r="G263" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A264" t="s">
+        <v>136</v>
+      </c>
+      <c r="B264" t="s">
+        <v>105</v>
+      </c>
+      <c r="C264" t="s">
+        <v>90</v>
+      </c>
+      <c r="D264">
+        <v>22</v>
+      </c>
+      <c r="E264">
+        <v>179</v>
+      </c>
+      <c r="F264" t="s">
+        <v>92</v>
+      </c>
+      <c r="G264" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A265" t="s">
+        <v>136</v>
+      </c>
+      <c r="B265" t="s">
+        <v>105</v>
+      </c>
+      <c r="C265" t="s">
+        <v>95</v>
+      </c>
+      <c r="D265">
+        <v>23</v>
+      </c>
+      <c r="E265">
+        <v>1</v>
+      </c>
+      <c r="F265" t="s">
+        <v>91</v>
+      </c>
+      <c r="G265" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A266" t="s">
+        <v>136</v>
+      </c>
+      <c r="B266" t="s">
+        <v>107</v>
+      </c>
+      <c r="C266" t="s">
+        <v>59</v>
+      </c>
+      <c r="D266">
+        <v>0</v>
+      </c>
+      <c r="E266">
+        <v>2</v>
+      </c>
+      <c r="F266" t="s">
+        <v>43</v>
+      </c>
+      <c r="G266" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A267" t="s">
+        <v>136</v>
+      </c>
+      <c r="B267" t="s">
+        <v>107</v>
+      </c>
+      <c r="C267" t="s">
+        <v>63</v>
+      </c>
+      <c r="D267">
+        <v>1</v>
+      </c>
+      <c r="E267">
+        <v>1</v>
+      </c>
+      <c r="F267" t="s">
+        <v>43</v>
+      </c>
+      <c r="G267" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
+        <v>136</v>
+      </c>
+      <c r="B268" t="s">
+        <v>107</v>
+      </c>
+      <c r="C268" t="s">
+        <v>54</v>
+      </c>
+      <c r="D268">
+        <v>2</v>
+      </c>
+      <c r="E268">
+        <v>2</v>
+      </c>
+      <c r="F268" t="s">
+        <v>43</v>
+      </c>
+      <c r="G268" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
+        <v>136</v>
+      </c>
+      <c r="B269" t="s">
+        <v>107</v>
+      </c>
+      <c r="C269" t="s">
+        <v>55</v>
+      </c>
+      <c r="D269">
+        <v>3</v>
+      </c>
+      <c r="E269">
+        <v>2</v>
+      </c>
+      <c r="F269" t="s">
+        <v>43</v>
+      </c>
+      <c r="G269" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
+        <v>136</v>
+      </c>
+      <c r="B270" t="s">
+        <v>107</v>
+      </c>
+      <c r="C270" t="s">
+        <v>56</v>
+      </c>
+      <c r="D270">
+        <v>4</v>
+      </c>
+      <c r="E270">
+        <v>2</v>
+      </c>
+      <c r="F270" t="s">
+        <v>43</v>
+      </c>
+      <c r="G270" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
+        <v>136</v>
+      </c>
+      <c r="B271" t="s">
+        <v>107</v>
+      </c>
+      <c r="C271" t="s">
+        <v>64</v>
+      </c>
+      <c r="D271">
+        <v>5</v>
+      </c>
+      <c r="E271">
+        <v>22000</v>
+      </c>
+      <c r="F271" t="s">
+        <v>41</v>
+      </c>
+      <c r="G271" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>136</v>
+      </c>
+      <c r="B272" t="s">
+        <v>107</v>
+      </c>
+      <c r="C272" t="s">
+        <v>61</v>
+      </c>
+      <c r="D272">
+        <v>6</v>
+      </c>
+      <c r="E272">
+        <v>0</v>
+      </c>
+      <c r="F272" t="s">
+        <v>42</v>
+      </c>
+      <c r="G272" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
+        <v>136</v>
+      </c>
+      <c r="B273" t="s">
+        <v>107</v>
+      </c>
+      <c r="C273" t="s">
+        <v>62</v>
+      </c>
+      <c r="D273">
+        <v>7</v>
+      </c>
+      <c r="E273">
+        <v>3</v>
+      </c>
+      <c r="F273" t="s">
+        <v>72</v>
+      </c>
+      <c r="G273" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
+        <v>136</v>
+      </c>
+      <c r="B274" t="s">
+        <v>107</v>
+      </c>
+      <c r="C274" t="s">
+        <v>65</v>
+      </c>
+      <c r="D274">
+        <v>8</v>
+      </c>
+      <c r="E274">
+        <v>0.06</v>
+      </c>
+      <c r="F274" t="s">
+        <v>42</v>
+      </c>
+      <c r="G274" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>136</v>
+      </c>
+      <c r="B275" t="s">
+        <v>107</v>
+      </c>
+      <c r="C275" t="s">
+        <v>58</v>
+      </c>
+      <c r="D275">
+        <v>9</v>
+      </c>
+      <c r="E275">
+        <v>1</v>
+      </c>
+      <c r="F275" t="s">
+        <v>43</v>
+      </c>
+      <c r="G275" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>136</v>
+      </c>
+      <c r="B276" t="s">
+        <v>107</v>
+      </c>
+      <c r="C276" t="s">
+        <v>60</v>
+      </c>
+      <c r="D276">
+        <v>10</v>
+      </c>
+      <c r="E276">
+        <v>1</v>
+      </c>
+      <c r="F276" t="s">
+        <v>43</v>
+      </c>
+      <c r="G276" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A277" t="s">
+        <v>136</v>
+      </c>
+      <c r="B277" t="s">
+        <v>107</v>
+      </c>
+      <c r="C277" t="s">
+        <v>57</v>
+      </c>
+      <c r="D277">
+        <v>11</v>
+      </c>
+      <c r="E277">
+        <v>1</v>
+      </c>
+      <c r="F277" t="s">
+        <v>43</v>
+      </c>
+      <c r="G277" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>136</v>
+      </c>
+      <c r="B278" t="s">
+        <v>107</v>
+      </c>
+      <c r="C278" t="s">
+        <v>40</v>
+      </c>
+      <c r="D278">
+        <v>12</v>
+      </c>
+      <c r="E278">
+        <v>0.7</v>
+      </c>
+      <c r="F278" t="s">
+        <v>43</v>
+      </c>
+      <c r="G278" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>136</v>
+      </c>
+      <c r="B279" t="s">
+        <v>107</v>
+      </c>
+      <c r="C279" t="s">
+        <v>70</v>
+      </c>
+      <c r="D279">
+        <v>13</v>
+      </c>
+      <c r="E279">
+        <v>16</v>
+      </c>
+      <c r="F279" t="s">
+        <v>44</v>
+      </c>
+      <c r="G279" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
+        <v>136</v>
+      </c>
+      <c r="B280" t="s">
+        <v>107</v>
+      </c>
+      <c r="C280" t="s">
+        <v>45</v>
+      </c>
+      <c r="D280">
+        <v>14</v>
+      </c>
+      <c r="E280">
+        <v>13</v>
+      </c>
+      <c r="F280" t="s">
+        <v>72</v>
+      </c>
+      <c r="G280" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
+        <v>136</v>
+      </c>
+      <c r="B281" t="s">
+        <v>107</v>
+      </c>
+      <c r="C281" t="s">
+        <v>53</v>
+      </c>
+      <c r="D281">
+        <v>15</v>
+      </c>
+      <c r="E281">
+        <v>13</v>
+      </c>
+      <c r="F281" t="s">
+        <v>72</v>
+      </c>
+      <c r="G281" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
+        <v>136</v>
+      </c>
+      <c r="B282" t="s">
+        <v>107</v>
+      </c>
+      <c r="C282" t="s">
+        <v>47</v>
+      </c>
+      <c r="D282">
+        <v>16</v>
+      </c>
+      <c r="E282">
+        <v>4</v>
+      </c>
+      <c r="F282" t="s">
+        <v>72</v>
+      </c>
+      <c r="G282" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
+        <v>136</v>
+      </c>
+      <c r="B283" t="s">
+        <v>107</v>
+      </c>
+      <c r="C283" t="s">
+        <v>48</v>
+      </c>
+      <c r="D283">
+        <v>17</v>
+      </c>
+      <c r="E283">
+        <v>3</v>
+      </c>
+      <c r="F283" t="s">
+        <v>72</v>
+      </c>
+      <c r="G283" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A284" t="s">
+        <v>136</v>
+      </c>
+      <c r="B284" t="s">
+        <v>107</v>
+      </c>
+      <c r="C284" t="s">
+        <v>49</v>
+      </c>
+      <c r="D284">
+        <v>18</v>
+      </c>
+      <c r="E284">
+        <v>5</v>
+      </c>
+      <c r="F284" t="s">
+        <v>72</v>
+      </c>
+      <c r="G284" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
+        <v>136</v>
+      </c>
+      <c r="B285" t="s">
+        <v>107</v>
+      </c>
+      <c r="C285" t="s">
+        <v>68</v>
+      </c>
+      <c r="D285">
+        <v>19</v>
+      </c>
+      <c r="E285">
+        <v>250000000</v>
+      </c>
+      <c r="F285" t="s">
+        <v>73</v>
+      </c>
+      <c r="G285" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>136</v>
+      </c>
+      <c r="B286" t="s">
+        <v>107</v>
+      </c>
+      <c r="C286" t="s">
+        <v>69</v>
+      </c>
+      <c r="D286">
+        <v>20</v>
+      </c>
+      <c r="E286">
+        <v>150000000</v>
+      </c>
+      <c r="F286" t="s">
+        <v>73</v>
+      </c>
+      <c r="G286" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
+        <v>136</v>
+      </c>
+      <c r="B287" t="s">
+        <v>107</v>
+      </c>
+      <c r="C287" t="s">
+        <v>89</v>
+      </c>
+      <c r="D287">
+        <v>21</v>
+      </c>
+      <c r="E287">
+        <v>13</v>
+      </c>
+      <c r="F287" t="s">
+        <v>91</v>
+      </c>
+      <c r="G287" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
+        <v>136</v>
+      </c>
+      <c r="B288" t="s">
+        <v>107</v>
+      </c>
+      <c r="C288" t="s">
+        <v>90</v>
+      </c>
+      <c r="D288">
+        <v>22</v>
+      </c>
+      <c r="E288">
+        <v>179</v>
+      </c>
+      <c r="F288" t="s">
+        <v>92</v>
+      </c>
+      <c r="G288" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>136</v>
+      </c>
+      <c r="B289" t="s">
+        <v>107</v>
+      </c>
+      <c r="C289" t="s">
+        <v>95</v>
+      </c>
+      <c r="D289">
+        <v>23</v>
+      </c>
+      <c r="E289">
+        <v>1</v>
+      </c>
+      <c r="F289" t="s">
+        <v>91</v>
+      </c>
+      <c r="G289" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A290" t="s">
+        <v>136</v>
+      </c>
+      <c r="B290" t="s">
+        <v>71</v>
+      </c>
+      <c r="C290" t="s">
+        <v>137</v>
+      </c>
+      <c r="D290">
+        <v>24</v>
+      </c>
+      <c r="E290">
+        <v>1</v>
+      </c>
+      <c r="F290" t="s">
+        <v>43</v>
+      </c>
+      <c r="G290" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
+        <v>136</v>
+      </c>
+      <c r="B291" t="s">
+        <v>88</v>
+      </c>
+      <c r="C291" t="s">
+        <v>137</v>
+      </c>
+      <c r="D291">
+        <v>24</v>
+      </c>
+      <c r="E291">
+        <v>1</v>
+      </c>
+      <c r="F291" t="s">
+        <v>43</v>
+      </c>
+      <c r="G291" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A292" t="s">
+        <v>136</v>
+      </c>
+      <c r="B292" t="s">
+        <v>87</v>
+      </c>
+      <c r="C292" t="s">
+        <v>137</v>
+      </c>
+      <c r="D292">
+        <v>24</v>
+      </c>
+      <c r="E292">
+        <v>1</v>
+      </c>
+      <c r="F292" t="s">
+        <v>43</v>
+      </c>
+      <c r="G292" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A293" t="s">
+        <v>136</v>
+      </c>
+      <c r="B293" t="s">
+        <v>106</v>
+      </c>
+      <c r="C293" t="s">
+        <v>137</v>
+      </c>
+      <c r="D293">
+        <v>24</v>
+      </c>
+      <c r="E293">
+        <v>1</v>
+      </c>
+      <c r="F293" t="s">
+        <v>43</v>
+      </c>
+      <c r="G293" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A294" t="s">
+        <v>136</v>
+      </c>
+      <c r="B294" t="s">
+        <v>105</v>
+      </c>
+      <c r="C294" t="s">
+        <v>137</v>
+      </c>
+      <c r="D294">
+        <v>24</v>
+      </c>
+      <c r="E294">
+        <v>1</v>
+      </c>
+      <c r="F294" t="s">
+        <v>43</v>
+      </c>
+      <c r="G294" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
+        <v>136</v>
+      </c>
+      <c r="B295" t="s">
+        <v>107</v>
+      </c>
+      <c r="C295" t="s">
+        <v>137</v>
+      </c>
+      <c r="D295">
+        <v>24</v>
+      </c>
+      <c r="E295">
+        <v>1</v>
+      </c>
+      <c r="F295" t="s">
+        <v>43</v>
+      </c>
+      <c r="G295" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>39</v>
+      </c>
+      <c r="B296" t="s">
+        <v>71</v>
+      </c>
+      <c r="C296" t="s">
+        <v>137</v>
+      </c>
+      <c r="D296">
+        <v>24</v>
+      </c>
+      <c r="E296">
+        <v>0</v>
+      </c>
+      <c r="F296" t="s">
+        <v>43</v>
+      </c>
+      <c r="G296" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
+        <v>39</v>
+      </c>
+      <c r="B297" t="s">
+        <v>88</v>
+      </c>
+      <c r="C297" t="s">
+        <v>137</v>
+      </c>
+      <c r="D297">
+        <v>24</v>
+      </c>
+      <c r="E297">
+        <v>0</v>
+      </c>
+      <c r="F297" t="s">
+        <v>43</v>
+      </c>
+      <c r="G297" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A298" t="s">
+        <v>39</v>
+      </c>
+      <c r="B298" t="s">
+        <v>87</v>
+      </c>
+      <c r="C298" t="s">
+        <v>137</v>
+      </c>
+      <c r="D298">
+        <v>24</v>
+      </c>
+      <c r="E298">
+        <v>0</v>
+      </c>
+      <c r="F298" t="s">
+        <v>43</v>
+      </c>
+      <c r="G298" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A299" t="s">
+        <v>39</v>
+      </c>
+      <c r="B299" t="s">
+        <v>106</v>
+      </c>
+      <c r="C299" t="s">
+        <v>137</v>
+      </c>
+      <c r="D299">
+        <v>24</v>
+      </c>
+      <c r="E299">
+        <v>0</v>
+      </c>
+      <c r="F299" t="s">
+        <v>43</v>
+      </c>
+      <c r="G299" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A300" t="s">
+        <v>39</v>
+      </c>
+      <c r="B300" t="s">
+        <v>105</v>
+      </c>
+      <c r="C300" t="s">
+        <v>137</v>
+      </c>
+      <c r="D300">
+        <v>24</v>
+      </c>
+      <c r="E300">
+        <v>0</v>
+      </c>
+      <c r="F300" t="s">
+        <v>43</v>
+      </c>
+      <c r="G300" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
+        <v>39</v>
+      </c>
+      <c r="B301" t="s">
+        <v>107</v>
+      </c>
+      <c r="C301" t="s">
+        <v>137</v>
+      </c>
+      <c r="D301">
+        <v>24</v>
+      </c>
+      <c r="E301">
+        <v>0</v>
+      </c>
+      <c r="F301" t="s">
+        <v>43</v>
+      </c>
+      <c r="G301" t="s">
+        <v>138</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G145" xr:uid="{9375A35C-8A58-4D70-9436-2E641DE51D25}"/>
+  <autoFilter ref="A1:G301" xr:uid="{9375A35C-8A58-4D70-9436-2E641DE51D25}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H237">
     <sortCondition ref="A2:A237"/>
     <sortCondition ref="B2:B237"/>
     <sortCondition ref="D2:D237"/>
   </sortState>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="90" verticalDpi="90" r:id="rId1"/>
 </worksheet>
@@ -5808,7 +10440,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08421A62-7A7F-4754-940E-DE21752714F2}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -5917,7 +10549,148 @@
         <v>73</v>
       </c>
     </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D9" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>103</v>
+      </c>
+      <c r="D14" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>136</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>135</v>
+      </c>
+      <c r="D15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>140</v>
+      </c>
+      <c r="D17" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:E15" xr:uid="{08421A62-7A7F-4754-940E-DE21752714F2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>